<commit_message>
feat(observability): add tenant job monitoring policies
</commit_message>
<xml_diff>
--- a/docs/test-data/test-full-coverage-import-suite/ta-tenant-config-package-test.xlsx
+++ b/docs/test-data/test-full-coverage-import-suite/ta-tenant-config-package-test.xlsx
@@ -1,23 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="resource_queue" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="business_calendar" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="batch_window" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="job_definition" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="file_channel_config" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="file_template_config" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pipeline_definition" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pipeline_step_definition" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="workflow_definition" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="workflow_node" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="workflow_edge" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="resource_queue" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="business_calendar" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="batch_window" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="job_definition" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="job_monitoring_policy" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="file_channel_config" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="file_template_config" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="pipeline_definition" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="pipeline_step_definition" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="workflow_definition" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="workflow_node" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="workflow_edge" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -729,6 +730,101 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>tenant_id</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>workflow_code</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>workflow_name</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>workflow_type</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>version</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>enabled</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>ta</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>TA_WF_SETTLEMENT</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>零售结算工作流</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>DAG</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>导入→核对→结算→导出</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:P5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1081,7 +1177,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2151,6 +2247,72 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>tenant_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>job_code</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>soft_runtime_seconds</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>soft_runtime_severity</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>start_grace_seconds</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>start_grace_severity</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>completion_deadline_local_time</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>completion_deadline_day_offset</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>completion_grace_seconds</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>completion_deadline_severity</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2373,7 +2535,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3492,7 +3654,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3699,7 +3861,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4651,99 +4813,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>tenant_id</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>workflow_code</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>workflow_name</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>workflow_type</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>version</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>enabled</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>ta</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>TA_WF_SETTLEMENT</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>零售结算工作流</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>DAG</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>导入→核对→结算→导出</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
feat(observability): add tenant job monitoring policies (#1199)
</commit_message>
<xml_diff>
--- a/docs/test-data/test-full-coverage-import-suite/ta-tenant-config-package-test.xlsx
+++ b/docs/test-data/test-full-coverage-import-suite/ta-tenant-config-package-test.xlsx
@@ -1,23 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="resource_queue" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="business_calendar" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="batch_window" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="job_definition" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="file_channel_config" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="file_template_config" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pipeline_definition" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pipeline_step_definition" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="workflow_definition" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="workflow_node" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="workflow_edge" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="resource_queue" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="business_calendar" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="batch_window" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="job_definition" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="job_monitoring_policy" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="file_channel_config" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="file_template_config" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="pipeline_definition" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="pipeline_step_definition" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="workflow_definition" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="workflow_node" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="workflow_edge" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -729,6 +730,101 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>tenant_id</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>workflow_code</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>workflow_name</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>workflow_type</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>version</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>enabled</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>ta</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>TA_WF_SETTLEMENT</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>零售结算工作流</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>DAG</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>导入→核对→结算→导出</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:P5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1081,7 +1177,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2151,6 +2247,72 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>tenant_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>job_code</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>soft_runtime_seconds</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>soft_runtime_severity</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>start_grace_seconds</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>start_grace_severity</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>completion_deadline_local_time</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>completion_deadline_day_offset</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>completion_grace_seconds</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>completion_deadline_severity</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2373,7 +2535,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3492,7 +3654,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3699,7 +3861,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4651,99 +4813,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>tenant_id</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>workflow_code</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>workflow_name</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>workflow_type</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>version</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>enabled</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>ta</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>TA_WF_SETTLEMENT</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>零售结算工作流</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>DAG</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>导入→核对→结算→导出</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
fix(sim): align tenant pipeline stage fixtures
</commit_message>
<xml_diff>
--- a/docs/test-data/test-full-coverage-import-suite/ta-tenant-config-package-test.xlsx
+++ b/docs/test-data/test-full-coverage-import-suite/ta-tenant-config-package-test.xlsx
@@ -3867,7 +3867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3971,7 +3971,7 @@
         </is>
       </c>
       <c r="F2" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
@@ -4025,7 +4025,7 @@
         </is>
       </c>
       <c r="F3" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
@@ -4079,7 +4079,7 @@
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
@@ -4133,7 +4133,7 @@
         </is>
       </c>
       <c r="F5" s="3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
@@ -4187,7 +4187,7 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -4241,7 +4241,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -4295,7 +4295,7 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -4349,7 +4349,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -4403,7 +4403,7 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -4457,7 +4457,7 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -4511,7 +4511,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -4565,7 +4565,7 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -4619,7 +4619,7 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -4673,7 +4673,7 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -4727,7 +4727,7 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -4781,7 +4781,7 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -4805,6 +4805,60 @@
         <v>0</v>
       </c>
       <c r="L17" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>TA_IMPORT_CUSTOMER</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>STEP_FEEDBACK</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>回执写回</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>FEEDBACK</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>5</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>IMPORT_FEEDBACK</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>120</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>

</xml_diff>

<commit_message>
fix(sim): align tenant pipeline stage fixtures (#1264)
Co-authored-by: Dengchao <tfys9544@gmail.com>
</commit_message>
<xml_diff>
--- a/docs/test-data/test-full-coverage-import-suite/ta-tenant-config-package-test.xlsx
+++ b/docs/test-data/test-full-coverage-import-suite/ta-tenant-config-package-test.xlsx
@@ -3867,7 +3867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3971,7 +3971,7 @@
         </is>
       </c>
       <c r="F2" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
@@ -4025,7 +4025,7 @@
         </is>
       </c>
       <c r="F3" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
@@ -4079,7 +4079,7 @@
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
@@ -4133,7 +4133,7 @@
         </is>
       </c>
       <c r="F5" s="3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
@@ -4187,7 +4187,7 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -4241,7 +4241,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -4295,7 +4295,7 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -4349,7 +4349,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -4403,7 +4403,7 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -4457,7 +4457,7 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -4511,7 +4511,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -4565,7 +4565,7 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -4619,7 +4619,7 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -4673,7 +4673,7 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -4727,7 +4727,7 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -4781,7 +4781,7 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -4805,6 +4805,60 @@
         <v>0</v>
       </c>
       <c r="L17" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>TA_IMPORT_CUSTOMER</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>STEP_FEEDBACK</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>回执写回</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>FEEDBACK</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>5</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>IMPORT_FEEDBACK</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>120</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>

</xml_diff>